<commit_message>
Add 11 more competitors to pricing research
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NoHsoyzsfNMbjZXdgBS5oa
</commit_message>
<xml_diff>
--- a/pricing/UFS_Pricing_Model.xlsx
+++ b/pricing/UFS_Pricing_Model.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="342">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="420">
   <si>
     <t xml:space="preserve">Client Fee Quote</t>
   </si>
@@ -518,7 +518,7 @@
     <t xml:space="preserve">Landlord (property only)</t>
   </si>
   <si>
-    <t xml:space="preserve">Hertfordshire competitor pricing research (gathered 23 Oct 2026 from public web pages)</t>
+    <t xml:space="preserve">Hertfordshire competitor pricing research (gathered 23–24 Oct 2026 from public web pages)</t>
   </si>
   <si>
     <t xml:space="preserve">Figures are advertised 'from' prices or published ranges, ex VAT unless stated. Not verified with the firms – treat as indicative and re-check before relying on them.</t>
@@ -881,6 +881,243 @@
     <t xml:space="preserve">https://www.bizhub365.com/find/accountant/watford/cost/</t>
   </si>
   <si>
+    <t xml:space="preserve">KE Accounting Solutions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stevenage / Hertfordshire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Local bookkeeping &amp; accounts firm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiered monthly packages by business size</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£400/m basic Ltd (no staff); £750/m multi-staff payroll; £1,500/m full AP/AR &amp; credit control</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hourly from £35/hr; entry packages from £150/m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Included in tiers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Xero/QuickBooks setup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Premium positioning – sells outsourced finance function, not compliance. Shows the ceiling of the local market.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://keaccountingsolutions.co.uk/hertfordshire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QK Accounts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beds / Herts / Bucks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Online/regional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bronze/Silver/Gold bundles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bronze £75/m (accounts, VAT, payroll up to 5); Silver £140/m; Gold £250/m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Standalone from £25/m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Standalone £150/qtr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Up to 5 staff in Bronze</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Free QuickBooks licence; Silver/Gold add monthly management meeting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Good-better-best tiers with a 'meeting' upsell. Bundling VAT+payroll makes standalone VAT (£150) look expensive.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.qkaccounts.com/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Connected Accounting (Bark)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Online, Xero partner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Two flat packages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£49/m + VAT (also landlords)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£99/m + VAT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Included</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not stated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simple two-price model, landlords priced same as sole traders.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.bark.com/en/gb/bookkeeping-services/hertfordshire/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hertford hourly bookkeeper</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hertford</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hourly, no contract</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£15/hr + VAT (Xero/QB/Sage)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No monthly contract</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low hourly rate – sets client expectation for basic data entry.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://bookkeepingservices.accountants/bookkeeping-services/hertford/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bishop's Stortford directory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bishop's Stortford</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Directory average</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entry monthly price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From £60/m + VAT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From £95/m + VAT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£150–£400/yr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Basic Ltd accounts £700–£1,200/yr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">East Herts entry prices sit above the online chains.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://businessfinancing.co.uk/accounting/bishops-stortford-accountants/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Landlord specialist</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Niche specialist</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monthly retainer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Landlords £100–£300/m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Niche specialists charge well above general firms – landlord niche worth considering.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://accountants-for-landlords.co.uk/near-me/hertfordshire-bishops-stortford/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mazuma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">National online</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monthly plans by turnover</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£98–£140/m + VAT (~£1,176/yr+)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">National online benchmark for a full Ltd package.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://taxroot.co.uk/blog/best-online-accountant-uk-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crunch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monthly subscription + one-off SA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From £27/m + VAT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not stated in source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£200 + VAT (rises near Jan deadline)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Software-led</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deadline surge pricing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Charging more for late SA work rewards early clients and covers January overtime.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aardvark Accounting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monthly package</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£89/m + VAT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TaxRoot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annual compliance-only</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From £389/yr (accounts, CT, CT600)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compliance-only pricing – the absolute floor for Ltd year-end.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Price Bailey</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Large regional chartered firm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bespoke quote</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Large firms don't publish prices – they compete on expertise and advisory.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.pricebailey.co.uk/locations/bishops-stortford/</t>
+  </si>
+  <si>
     <t xml:space="preserve">UFS prices vs Hertfordshire market (ex VAT)</t>
   </si>
   <si>
@@ -993,9 +1230,6 @@
   </si>
   <si>
     <t xml:space="preserve">Firm / model</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Monthly package</t>
   </si>
   <si>
     <t xml:space="preserve">Bookkeeping /yr</t>
@@ -3470,7 +3704,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M17"/>
+  <dimension ref="A1:M28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -4057,6 +4291,443 @@
       </c>
       <c r="M17" s="25" t="s">
         <v>284</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="25" t="s">
+        <v>285</v>
+      </c>
+      <c r="B18" s="25" t="s">
+        <v>286</v>
+      </c>
+      <c r="C18" s="25" t="s">
+        <v>287</v>
+      </c>
+      <c r="D18" s="25" t="s">
+        <v>288</v>
+      </c>
+      <c r="E18" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="F18" s="25" t="s">
+        <v>289</v>
+      </c>
+      <c r="G18" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="H18" s="25" t="s">
+        <v>290</v>
+      </c>
+      <c r="I18" s="25" t="s">
+        <v>291</v>
+      </c>
+      <c r="J18" s="25" t="s">
+        <v>291</v>
+      </c>
+      <c r="K18" s="25" t="s">
+        <v>292</v>
+      </c>
+      <c r="L18" s="25" t="s">
+        <v>293</v>
+      </c>
+      <c r="M18" s="25" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="25" t="s">
+        <v>295</v>
+      </c>
+      <c r="B19" s="25" t="s">
+        <v>296</v>
+      </c>
+      <c r="C19" s="25" t="s">
+        <v>297</v>
+      </c>
+      <c r="D19" s="25" t="s">
+        <v>298</v>
+      </c>
+      <c r="E19" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="F19" s="25" t="s">
+        <v>299</v>
+      </c>
+      <c r="G19" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="H19" s="25" t="s">
+        <v>300</v>
+      </c>
+      <c r="I19" s="25" t="s">
+        <v>301</v>
+      </c>
+      <c r="J19" s="25" t="s">
+        <v>302</v>
+      </c>
+      <c r="K19" s="25" t="s">
+        <v>303</v>
+      </c>
+      <c r="L19" s="25" t="s">
+        <v>304</v>
+      </c>
+      <c r="M19" s="25" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="25" t="s">
+        <v>306</v>
+      </c>
+      <c r="B20" s="25" t="s">
+        <v>241</v>
+      </c>
+      <c r="C20" s="25" t="s">
+        <v>307</v>
+      </c>
+      <c r="D20" s="25" t="s">
+        <v>308</v>
+      </c>
+      <c r="E20" s="25" t="s">
+        <v>309</v>
+      </c>
+      <c r="F20" s="25" t="s">
+        <v>310</v>
+      </c>
+      <c r="G20" s="25" t="s">
+        <v>311</v>
+      </c>
+      <c r="H20" s="25" t="s">
+        <v>312</v>
+      </c>
+      <c r="I20" s="25" t="s">
+        <v>312</v>
+      </c>
+      <c r="J20" s="25" t="s">
+        <v>312</v>
+      </c>
+      <c r="K20" s="25"/>
+      <c r="L20" s="25" t="s">
+        <v>313</v>
+      </c>
+      <c r="M20" s="25" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="25" t="s">
+        <v>315</v>
+      </c>
+      <c r="B21" s="25" t="s">
+        <v>316</v>
+      </c>
+      <c r="C21" s="25" t="s">
+        <v>228</v>
+      </c>
+      <c r="D21" s="25" t="s">
+        <v>317</v>
+      </c>
+      <c r="E21" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="F21" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="G21" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="H21" s="25" t="s">
+        <v>318</v>
+      </c>
+      <c r="I21" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="J21" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="K21" s="25" t="s">
+        <v>319</v>
+      </c>
+      <c r="L21" s="25" t="s">
+        <v>320</v>
+      </c>
+      <c r="M21" s="25" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="25" t="s">
+        <v>322</v>
+      </c>
+      <c r="B22" s="25" t="s">
+        <v>323</v>
+      </c>
+      <c r="C22" s="25" t="s">
+        <v>324</v>
+      </c>
+      <c r="D22" s="25" t="s">
+        <v>325</v>
+      </c>
+      <c r="E22" s="25" t="s">
+        <v>326</v>
+      </c>
+      <c r="F22" s="25" t="s">
+        <v>327</v>
+      </c>
+      <c r="G22" s="25" t="s">
+        <v>328</v>
+      </c>
+      <c r="H22" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="I22" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="J22" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="K22" s="25" t="s">
+        <v>329</v>
+      </c>
+      <c r="L22" s="25" t="s">
+        <v>330</v>
+      </c>
+      <c r="M22" s="25" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="25" t="s">
+        <v>332</v>
+      </c>
+      <c r="B23" s="25" t="s">
+        <v>323</v>
+      </c>
+      <c r="C23" s="25" t="s">
+        <v>333</v>
+      </c>
+      <c r="D23" s="25" t="s">
+        <v>334</v>
+      </c>
+      <c r="E23" s="25" t="s">
+        <v>335</v>
+      </c>
+      <c r="F23" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="G23" s="25" t="s">
+        <v>311</v>
+      </c>
+      <c r="H23" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="I23" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="J23" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="K23" s="25"/>
+      <c r="L23" s="25" t="s">
+        <v>336</v>
+      </c>
+      <c r="M23" s="25" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="25" t="s">
+        <v>338</v>
+      </c>
+      <c r="B24" s="25" t="s">
+        <v>339</v>
+      </c>
+      <c r="C24" s="25" t="s">
+        <v>214</v>
+      </c>
+      <c r="D24" s="25" t="s">
+        <v>340</v>
+      </c>
+      <c r="E24" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="F24" s="25" t="s">
+        <v>341</v>
+      </c>
+      <c r="G24" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="H24" s="25" t="s">
+        <v>311</v>
+      </c>
+      <c r="I24" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="J24" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="K24" s="25"/>
+      <c r="L24" s="25" t="s">
+        <v>342</v>
+      </c>
+      <c r="M24" s="25" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="25" t="s">
+        <v>344</v>
+      </c>
+      <c r="B25" s="25" t="s">
+        <v>339</v>
+      </c>
+      <c r="C25" s="25" t="s">
+        <v>214</v>
+      </c>
+      <c r="D25" s="25" t="s">
+        <v>345</v>
+      </c>
+      <c r="E25" s="25" t="s">
+        <v>346</v>
+      </c>
+      <c r="F25" s="25" t="s">
+        <v>347</v>
+      </c>
+      <c r="G25" s="25" t="s">
+        <v>348</v>
+      </c>
+      <c r="H25" s="25" t="s">
+        <v>349</v>
+      </c>
+      <c r="I25" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="J25" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="K25" s="25" t="s">
+        <v>350</v>
+      </c>
+      <c r="L25" s="25" t="s">
+        <v>351</v>
+      </c>
+      <c r="M25" s="25" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="25" t="s">
+        <v>352</v>
+      </c>
+      <c r="B26" s="25" t="s">
+        <v>339</v>
+      </c>
+      <c r="C26" s="25" t="s">
+        <v>214</v>
+      </c>
+      <c r="D26" s="25" t="s">
+        <v>353</v>
+      </c>
+      <c r="E26" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="F26" s="25" t="s">
+        <v>354</v>
+      </c>
+      <c r="G26" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="H26" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="I26" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="J26" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="K26" s="25"/>
+      <c r="L26" s="25"/>
+      <c r="M26" s="25" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="25" t="s">
+        <v>355</v>
+      </c>
+      <c r="B27" s="25" t="s">
+        <v>339</v>
+      </c>
+      <c r="C27" s="25" t="s">
+        <v>214</v>
+      </c>
+      <c r="D27" s="25" t="s">
+        <v>356</v>
+      </c>
+      <c r="E27" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="F27" s="25" t="s">
+        <v>357</v>
+      </c>
+      <c r="G27" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="H27" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="I27" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="J27" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="K27" s="25"/>
+      <c r="L27" s="25" t="s">
+        <v>358</v>
+      </c>
+      <c r="M27" s="25" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="25" t="s">
+        <v>359</v>
+      </c>
+      <c r="B28" s="25" t="s">
+        <v>323</v>
+      </c>
+      <c r="C28" s="25" t="s">
+        <v>360</v>
+      </c>
+      <c r="D28" s="25" t="s">
+        <v>361</v>
+      </c>
+      <c r="E28" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="F28" s="25" t="s">
+        <v>182</v>
+      </c>
+      <c r="G28" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="H28" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="I28" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="J28" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="K28" s="25"/>
+      <c r="L28" s="25" t="s">
+        <v>362</v>
+      </c>
+      <c r="M28" s="25" t="s">
+        <v>363</v>
       </c>
     </row>
   </sheetData>
@@ -4090,12 +4761,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="22" t="s">
-        <v>285</v>
+        <v>364</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="23" t="s">
-        <v>286</v>
+        <v>365</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4103,33 +4774,33 @@
         <v>39</v>
       </c>
       <c r="B4" s="24" t="s">
-        <v>287</v>
+        <v>366</v>
       </c>
       <c r="C4" s="24" t="s">
-        <v>288</v>
+        <v>367</v>
       </c>
       <c r="D4" s="24" t="s">
-        <v>289</v>
+        <v>368</v>
       </c>
       <c r="E4" s="24" t="s">
-        <v>290</v>
+        <v>369</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>291</v>
+        <v>370</v>
       </c>
       <c r="G4" s="24" t="s">
-        <v>292</v>
+        <v>371</v>
       </c>
       <c r="H4" s="24" t="s">
-        <v>293</v>
+        <v>372</v>
       </c>
       <c r="I4" s="24" t="s">
-        <v>294</v>
+        <v>373</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="s">
-        <v>295</v>
+        <v>374</v>
       </c>
       <c r="B5" s="26" t="s">
         <v>101</v>
@@ -4156,12 +4827,12 @@
         <v>0.00502512562814061</v>
       </c>
       <c r="I5" s="25" t="s">
-        <v>296</v>
+        <v>375</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="26" t="s">
-        <v>297</v>
+        <v>376</v>
       </c>
       <c r="B6" s="26" t="s">
         <v>101</v>
@@ -4188,12 +4859,12 @@
         <v>0.104417670682731</v>
       </c>
       <c r="I6" s="25" t="s">
-        <v>298</v>
+        <v>377</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="26" t="s">
-        <v>299</v>
+        <v>378</v>
       </c>
       <c r="B7" s="26" t="s">
         <v>104</v>
@@ -4220,12 +4891,12 @@
         <v>0</v>
       </c>
       <c r="I7" s="25" t="s">
-        <v>300</v>
+        <v>379</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="26" t="s">
-        <v>301</v>
+        <v>380</v>
       </c>
       <c r="B8" s="26" t="s">
         <v>104</v>
@@ -4252,15 +4923,15 @@
         <v>0.0588235294117647</v>
       </c>
       <c r="I8" s="25" t="s">
-        <v>302</v>
+        <v>381</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="26" t="s">
-        <v>303</v>
+        <v>382</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>304</v>
+        <v>383</v>
       </c>
       <c r="C9" s="27" t="n">
         <v>75</v>
@@ -4284,15 +4955,15 @@
         <v>-0.25</v>
       </c>
       <c r="I9" s="25" t="s">
-        <v>305</v>
+        <v>384</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="26" t="s">
-        <v>306</v>
+        <v>385</v>
       </c>
       <c r="B10" s="26" t="s">
-        <v>307</v>
+        <v>386</v>
       </c>
       <c r="C10" s="27" t="n">
         <v>5</v>
@@ -4316,12 +4987,12 @@
         <v>-0.5</v>
       </c>
       <c r="I10" s="25" t="s">
-        <v>308</v>
+        <v>387</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="26" t="s">
-        <v>309</v>
+        <v>388</v>
       </c>
       <c r="B11" s="26" t="s">
         <v>92</v>
@@ -4348,12 +5019,12 @@
         <v>-0.6</v>
       </c>
       <c r="I11" s="25" t="s">
-        <v>310</v>
+        <v>389</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="26" t="s">
-        <v>311</v>
+        <v>390</v>
       </c>
       <c r="B12" s="26" t="s">
         <v>104</v>
@@ -4380,12 +5051,12 @@
         <v>0</v>
       </c>
       <c r="I12" s="25" t="s">
-        <v>312</v>
+        <v>391</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="26" t="s">
-        <v>313</v>
+        <v>392</v>
       </c>
       <c r="B13" s="26" t="s">
         <v>92</v>
@@ -4412,12 +5083,12 @@
         <v>-0.240506329113924</v>
       </c>
       <c r="I13" s="25" t="s">
-        <v>314</v>
+        <v>393</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="26" t="s">
-        <v>315</v>
+        <v>394</v>
       </c>
       <c r="B14" s="26" t="s">
         <v>92</v>
@@ -4444,12 +5115,12 @@
         <v>-0.536</v>
       </c>
       <c r="I14" s="25" t="s">
-        <v>316</v>
+        <v>395</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="26" t="s">
-        <v>317</v>
+        <v>396</v>
       </c>
       <c r="B15" s="26" t="s">
         <v>141</v>
@@ -4476,7 +5147,7 @@
         <v>-0.1</v>
       </c>
       <c r="I15" s="25" t="s">
-        <v>318</v>
+        <v>397</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4508,7 +5179,7 @@
         <v>0</v>
       </c>
       <c r="I16" s="25" t="s">
-        <v>319</v>
+        <v>398</v>
       </c>
     </row>
   </sheetData>
@@ -4539,12 +5210,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="22" t="s">
-        <v>320</v>
+        <v>399</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="30" t="s">
-        <v>321</v>
+        <v>400</v>
       </c>
       <c r="B2" s="30"/>
       <c r="C2" s="30"/>
@@ -4556,33 +5227,33 @@
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="24" t="s">
-        <v>322</v>
+        <v>401</v>
       </c>
       <c r="B4" s="24" t="s">
-        <v>323</v>
+        <v>353</v>
       </c>
       <c r="C4" s="24" t="s">
-        <v>324</v>
+        <v>402</v>
       </c>
       <c r="D4" s="24" t="s">
-        <v>325</v>
+        <v>403</v>
       </c>
       <c r="E4" s="24" t="s">
-        <v>326</v>
+        <v>404</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>327</v>
+        <v>405</v>
       </c>
       <c r="G4" s="24" t="s">
-        <v>328</v>
+        <v>406</v>
       </c>
       <c r="H4" s="24" t="s">
-        <v>329</v>
+        <v>407</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="31" t="s">
-        <v>330</v>
+        <v>408</v>
       </c>
       <c r="B5" s="32"/>
       <c r="C5" s="32"/>
@@ -4594,12 +5265,12 @@
         <v>5313.3</v>
       </c>
       <c r="H5" s="26" t="s">
-        <v>331</v>
+        <v>409</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="26" t="s">
-        <v>332</v>
+        <v>410</v>
       </c>
       <c r="B6" s="27" t="n">
         <v>480</v>
@@ -4625,12 +5296,12 @@
         <v>2826</v>
       </c>
       <c r="H6" s="26" t="s">
-        <v>333</v>
+        <v>411</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="26" t="s">
-        <v>334</v>
+        <v>412</v>
       </c>
       <c r="B7" s="27" t="n">
         <v>240</v>
@@ -4656,12 +5327,12 @@
         <v>2586</v>
       </c>
       <c r="H7" s="26" t="s">
-        <v>335</v>
+        <v>413</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="26" t="s">
-        <v>336</v>
+        <v>414</v>
       </c>
       <c r="B8" s="27" t="n">
         <v>0</v>
@@ -4687,12 +5358,12 @@
         <v>3150</v>
       </c>
       <c r="H8" s="26" t="s">
-        <v>337</v>
+        <v>415</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="26" t="s">
-        <v>338</v>
+        <v>416</v>
       </c>
       <c r="B9" s="27" t="n">
         <v>0</v>
@@ -4718,12 +5389,12 @@
         <v>3446</v>
       </c>
       <c r="H9" s="26" t="s">
-        <v>339</v>
+        <v>417</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="31" t="s">
-        <v>340</v>
+        <v>418</v>
       </c>
       <c r="G11" s="33" t="n">
         <f aca="false">G5-MIN(G6:G9)</f>
@@ -4732,7 +5403,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="23" t="s">
-        <v>341</v>
+        <v>419</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Merit Accountants billed prices to competitor research and market comparison
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NoHsoyzsfNMbjZXdgBS5oa
</commit_message>
<xml_diff>
--- a/pricing/UFS_Pricing_Model.xlsx
+++ b/pricing/UFS_Pricing_Model.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="809" uniqueCount="533">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="828" uniqueCount="546">
   <si>
     <t xml:space="preserve">Client Fee Quote</t>
   </si>
@@ -1443,6 +1443,36 @@
     <t xml:space="preserve">Compliance-only pricing – the absolute floor for Ltd year-end.</t>
   </si>
   <si>
+    <t xml:space="preserve">Merit Accountants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unknown (real invoices supplied by George)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Practice – actual bills, not advertised</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per-job invoicing, ex VAT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annual accounts £1,250 (2023), £1,200 (2024)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£200 per return (2023/24)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£350 one-off for a whole tax year of payroll</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Company formation (Companies House + HMRC) £150</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Real billed prices – more reliable than advertised 'from' prices. Accounts at £1,200–£1,250 sit above the Herts typical; payroll as one annual fee is simple to sell.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Client bills dated Feb 2025 – Apr 2026 (screenshots)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Price Bailey</t>
   </si>
   <si>
@@ -1491,7 +1521,7 @@
     <t xml:space="preserve">Self assessment – simple</t>
   </si>
   <si>
-    <t xml:space="preserve">£136 all-in / £199 x3 local firms / guide £150–£400</t>
+    <t xml:space="preserve">£136 all-in / £199 x3 local firms / Merit £200 billed / guide £150–£400</t>
   </si>
   <si>
     <t xml:space="preserve">Self assessment – landlord (1 property)</t>
@@ -1503,7 +1533,7 @@
     <t xml:space="preserve">Ltd accounts + CT600 (turnover £90k–£250k)</t>
   </si>
   <si>
-    <t xml:space="preserve">Herts/Hemel guide £750–£2,000; Herts Accountants £500–£1,500 accounts only</t>
+    <t xml:space="preserve">Herts/Hemel guide £750–£2,000; Herts Accountants £500–£1,500 accounts only; Merit Accountants billed £1,200–£1,250 for accounts</t>
   </si>
   <si>
     <t xml:space="preserve">Ltd accounts + CT600 (under £90k)</t>
@@ -1552,6 +1582,15 @@
   </si>
   <si>
     <t xml:space="preserve">Guide £100–£500/m. UFS figure = base + 120 tx/month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Payroll – annual fee, small company</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Merit Accountants billed £350 for a full tax year; UK firm £375/yr for 1–5 staff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Merit Accountants billed £150; FCLS £153 inc VAT (~£128 ex)</t>
   </si>
   <si>
     <t xml:space="preserve">Ad hoc / advisory</t>
@@ -6310,7 +6349,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M28"/>
+  <dimension ref="A1:M29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -7297,43 +7336,84 @@
         <v>456</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="27" t="s">
         <v>472</v>
       </c>
       <c r="B28" s="27" t="s">
+        <v>473</v>
+      </c>
+      <c r="C28" s="27" t="s">
+        <v>474</v>
+      </c>
+      <c r="D28" s="27" t="s">
+        <v>475</v>
+      </c>
+      <c r="E28" s="27" t="s">
+        <v>314</v>
+      </c>
+      <c r="F28" s="27" t="s">
+        <v>476</v>
+      </c>
+      <c r="G28" s="27" t="s">
+        <v>477</v>
+      </c>
+      <c r="H28" s="27" t="s">
+        <v>314</v>
+      </c>
+      <c r="I28" s="27" t="s">
+        <v>314</v>
+      </c>
+      <c r="J28" s="27" t="s">
+        <v>478</v>
+      </c>
+      <c r="K28" s="27" t="s">
+        <v>479</v>
+      </c>
+      <c r="L28" s="27" t="s">
+        <v>480</v>
+      </c>
+      <c r="M28" s="27" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="27" t="s">
+        <v>482</v>
+      </c>
+      <c r="B29" s="27" t="s">
         <v>436</v>
       </c>
-      <c r="C28" s="27" t="s">
-        <v>473</v>
-      </c>
-      <c r="D28" s="27" t="s">
-        <v>474</v>
-      </c>
-      <c r="E28" s="27" t="s">
-        <v>314</v>
-      </c>
-      <c r="F28" s="27" t="s">
+      <c r="C29" s="27" t="s">
+        <v>483</v>
+      </c>
+      <c r="D29" s="27" t="s">
+        <v>484</v>
+      </c>
+      <c r="E29" s="27" t="s">
+        <v>314</v>
+      </c>
+      <c r="F29" s="27" t="s">
         <v>295</v>
       </c>
-      <c r="G28" s="27" t="s">
-        <v>314</v>
-      </c>
-      <c r="H28" s="27" t="s">
-        <v>314</v>
-      </c>
-      <c r="I28" s="27" t="s">
-        <v>314</v>
-      </c>
-      <c r="J28" s="27" t="s">
-        <v>314</v>
-      </c>
-      <c r="K28" s="27"/>
-      <c r="L28" s="27" t="s">
-        <v>475</v>
-      </c>
-      <c r="M28" s="27" t="s">
-        <v>476</v>
+      <c r="G29" s="27" t="s">
+        <v>314</v>
+      </c>
+      <c r="H29" s="27" t="s">
+        <v>314</v>
+      </c>
+      <c r="I29" s="27" t="s">
+        <v>314</v>
+      </c>
+      <c r="J29" s="27" t="s">
+        <v>314</v>
+      </c>
+      <c r="K29" s="27"/>
+      <c r="L29" s="27" t="s">
+        <v>485</v>
+      </c>
+      <c r="M29" s="27" t="s">
+        <v>486</v>
       </c>
     </row>
   </sheetData>
@@ -7352,7 +7432,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
@@ -7367,12 +7447,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>477</v>
+        <v>487</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>478</v>
+        <v>488</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7380,33 +7460,33 @@
         <v>39</v>
       </c>
       <c r="B4" s="26" t="s">
-        <v>479</v>
+        <v>489</v>
       </c>
       <c r="C4" s="26" t="s">
-        <v>480</v>
+        <v>490</v>
       </c>
       <c r="D4" s="26" t="s">
-        <v>481</v>
+        <v>491</v>
       </c>
       <c r="E4" s="26" t="s">
-        <v>482</v>
+        <v>492</v>
       </c>
       <c r="F4" s="26" t="s">
-        <v>483</v>
+        <v>493</v>
       </c>
       <c r="G4" s="26" t="s">
-        <v>484</v>
+        <v>494</v>
       </c>
       <c r="H4" s="26" t="s">
-        <v>485</v>
+        <v>495</v>
       </c>
       <c r="I4" s="26" t="s">
-        <v>486</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>487</v>
+        <v>497</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>103</v>
@@ -7433,12 +7513,12 @@
         <v>0.00502512562814061</v>
       </c>
       <c r="I5" s="27" t="s">
-        <v>488</v>
+        <v>498</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>489</v>
+        <v>499</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>103</v>
@@ -7465,12 +7545,12 @@
         <v>0.104417670682731</v>
       </c>
       <c r="I6" s="27" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>491</v>
+        <v>501</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>106</v>
@@ -7497,12 +7577,12 @@
         <v>0</v>
       </c>
       <c r="I7" s="27" t="s">
-        <v>492</v>
+        <v>502</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>493</v>
+        <v>503</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>106</v>
@@ -7529,15 +7609,15 @@
         <v>0.0588235294117647</v>
       </c>
       <c r="I8" s="27" t="s">
-        <v>494</v>
+        <v>504</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>495</v>
+        <v>505</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>496</v>
+        <v>506</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>75</v>
@@ -7561,15 +7641,15 @@
         <v>-0.25</v>
       </c>
       <c r="I9" s="27" t="s">
-        <v>497</v>
+        <v>507</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>498</v>
+        <v>508</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>499</v>
+        <v>509</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>5</v>
@@ -7593,12 +7673,12 @@
         <v>-0.5</v>
       </c>
       <c r="I10" s="27" t="s">
-        <v>500</v>
+        <v>510</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>501</v>
+        <v>511</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>94</v>
@@ -7625,12 +7705,12 @@
         <v>-0.6</v>
       </c>
       <c r="I11" s="27" t="s">
-        <v>502</v>
+        <v>512</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>503</v>
+        <v>513</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>106</v>
@@ -7657,12 +7737,12 @@
         <v>0</v>
       </c>
       <c r="I12" s="27" t="s">
-        <v>504</v>
+        <v>514</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>505</v>
+        <v>515</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>94</v>
@@ -7689,12 +7769,12 @@
         <v>-0.240506329113924</v>
       </c>
       <c r="I13" s="27" t="s">
-        <v>506</v>
+        <v>516</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>507</v>
+        <v>517</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>94</v>
@@ -7721,28 +7801,28 @@
         <v>-0.536</v>
       </c>
       <c r="I14" s="27" t="s">
-        <v>508</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>509</v>
+        <v>519</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>143</v>
+        <v>106</v>
       </c>
       <c r="C15" s="28" t="n">
-        <v>50</v>
+        <v>240</v>
       </c>
       <c r="D15" s="28" t="n">
-        <v>100</v>
+        <v>350</v>
       </c>
       <c r="E15" s="28" t="n">
-        <v>200</v>
+        <v>600</v>
       </c>
       <c r="F15" s="29" t="n">
-        <f aca="false">'Rate Card'!$B$45</f>
-        <v>90</v>
+        <f aca="false">12*'Rate Card'!$B$18</f>
+        <v>240</v>
       </c>
       <c r="G15" s="6" t="str">
         <f aca="false">IF(F15&lt;C15,"Below market",IF(F15&gt;E15,"Above market",IF(F15&lt;D15,"Low end of range","High end of range")))</f>
@@ -7750,31 +7830,31 @@
       </c>
       <c r="H15" s="30" t="n">
         <f aca="false">IF(D15=0,0,F15/D15-1)</f>
-        <v>-0.1</v>
+        <v>-0.314285714285714</v>
       </c>
       <c r="I15" s="27" t="s">
-        <v>510</v>
+        <v>520</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>108</v>
       </c>
       <c r="C16" s="28" t="n">
-        <v>350</v>
+        <v>128</v>
       </c>
       <c r="D16" s="28" t="n">
-        <v>450</v>
+        <v>150</v>
       </c>
       <c r="E16" s="28" t="n">
-        <v>630</v>
+        <v>195</v>
       </c>
       <c r="F16" s="29" t="n">
-        <f aca="false">'Rate Card'!$B$41</f>
-        <v>450</v>
+        <f aca="false">'Rate Card'!$B$40</f>
+        <v>150</v>
       </c>
       <c r="G16" s="6" t="str">
         <f aca="false">IF(F16&lt;C16,"Below market",IF(F16&gt;E16,"Above market",IF(F16&lt;D16,"Low end of range","High end of range")))</f>
@@ -7785,7 +7865,71 @@
         <v>0</v>
       </c>
       <c r="I16" s="27" t="s">
-        <v>511</v>
+        <v>521</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="s">
+        <v>522</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="C17" s="28" t="n">
+        <v>50</v>
+      </c>
+      <c r="D17" s="28" t="n">
+        <v>100</v>
+      </c>
+      <c r="E17" s="28" t="n">
+        <v>200</v>
+      </c>
+      <c r="F17" s="29" t="n">
+        <f aca="false">'Rate Card'!$B$45</f>
+        <v>90</v>
+      </c>
+      <c r="G17" s="6" t="str">
+        <f aca="false">IF(F17&lt;C17,"Below market",IF(F17&gt;E17,"Above market",IF(F17&lt;D17,"Low end of range","High end of range")))</f>
+        <v>Low end of range</v>
+      </c>
+      <c r="H17" s="30" t="n">
+        <f aca="false">IF(D17=0,0,F17/D17-1)</f>
+        <v>-0.1</v>
+      </c>
+      <c r="I17" s="27" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="C18" s="28" t="n">
+        <v>350</v>
+      </c>
+      <c r="D18" s="28" t="n">
+        <v>450</v>
+      </c>
+      <c r="E18" s="28" t="n">
+        <v>630</v>
+      </c>
+      <c r="F18" s="29" t="n">
+        <f aca="false">'Rate Card'!$B$41</f>
+        <v>450</v>
+      </c>
+      <c r="G18" s="6" t="str">
+        <f aca="false">IF(F18&lt;C18,"Below market",IF(F18&gt;E18,"Above market",IF(F18&lt;D18,"Low end of range","High end of range")))</f>
+        <v>High end of range</v>
+      </c>
+      <c r="H18" s="30" t="n">
+        <f aca="false">IF(D18=0,0,F18/D18-1)</f>
+        <v>0</v>
+      </c>
+      <c r="I18" s="27" t="s">
+        <v>524</v>
       </c>
     </row>
   </sheetData>
@@ -7816,12 +7960,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>512</v>
+        <v>525</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="31" t="s">
-        <v>513</v>
+        <v>526</v>
       </c>
       <c r="B2" s="31"/>
       <c r="C2" s="31"/>
@@ -7833,33 +7977,33 @@
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="26" t="s">
-        <v>514</v>
+        <v>527</v>
       </c>
       <c r="B4" s="26" t="s">
         <v>466</v>
       </c>
       <c r="C4" s="26" t="s">
-        <v>515</v>
+        <v>528</v>
       </c>
       <c r="D4" s="26" t="s">
-        <v>516</v>
+        <v>529</v>
       </c>
       <c r="E4" s="26" t="s">
-        <v>517</v>
+        <v>530</v>
       </c>
       <c r="F4" s="26" t="s">
-        <v>518</v>
+        <v>531</v>
       </c>
       <c r="G4" s="26" t="s">
-        <v>519</v>
+        <v>532</v>
       </c>
       <c r="H4" s="26" t="s">
-        <v>520</v>
+        <v>533</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>521</v>
+        <v>534</v>
       </c>
       <c r="B5" s="32"/>
       <c r="C5" s="32"/>
@@ -7871,12 +8015,12 @@
         <v>5313.3</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>522</v>
+        <v>535</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>523</v>
+        <v>536</v>
       </c>
       <c r="B6" s="28" t="n">
         <v>480</v>
@@ -7902,12 +8046,12 @@
         <v>2826</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>524</v>
+        <v>537</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>525</v>
+        <v>538</v>
       </c>
       <c r="B7" s="28" t="n">
         <v>240</v>
@@ -7933,12 +8077,12 @@
         <v>2586</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>526</v>
+        <v>539</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>527</v>
+        <v>540</v>
       </c>
       <c r="B8" s="28" t="n">
         <v>0</v>
@@ -7964,12 +8108,12 @@
         <v>3150</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>528</v>
+        <v>541</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>529</v>
+        <v>542</v>
       </c>
       <c r="B9" s="28" t="n">
         <v>0</v>
@@ -7995,12 +8139,12 @@
         <v>3446</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>530</v>
+        <v>543</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>531</v>
+        <v>544</v>
       </c>
       <c r="G11" s="33" t="n">
         <f aca="false">G5-MIN(G6:G9)</f>
@@ -8009,7 +8153,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>532</v>
+        <v>545</v>
       </c>
     </row>
   </sheetData>

</xml_diff>